<commit_message>
Update price tables -marzo
</commit_message>
<xml_diff>
--- a/cotizador.xlsx
+++ b/cotizador.xlsx
@@ -162,7 +162,7 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" shrinkToFit="1"/>
     </xf>
-    <xf numFmtId="164" fontId="2" fillId="0" borderId="0" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -490,25 +490,25 @@
         <v>7</v>
       </c>
       <c r="B2" s="3">
-        <v>100060</v>
+        <v>102962</v>
       </c>
       <c r="C2" s="3">
-        <v>128519</v>
+        <v>132246</v>
       </c>
       <c r="D2" s="3">
-        <v>169134</v>
+        <v>174039</v>
       </c>
       <c r="E2" s="3">
-        <v>286730</v>
+        <v>295045</v>
       </c>
       <c r="F2" s="3">
-        <v>494971</v>
+        <v>509325</v>
       </c>
       <c r="G2" s="3">
-        <v>87146</v>
+        <v>89673</v>
       </c>
       <c r="H2" s="3">
-        <v>75170</v>
+        <v>77350</v>
       </c>
     </row>
     <row r="3" spans="1:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
@@ -516,25 +516,25 @@
         <v>8</v>
       </c>
       <c r="B3" s="3">
-        <v>100496</v>
+        <v>103410</v>
       </c>
       <c r="C3" s="3">
-        <v>138170</v>
+        <v>142177</v>
       </c>
       <c r="D3" s="3">
-        <v>170735</v>
+        <v>175686</v>
       </c>
       <c r="E3" s="3">
-        <v>294623</v>
+        <v>303167</v>
       </c>
       <c r="F3" s="3">
-        <v>496503</v>
+        <v>510902</v>
       </c>
       <c r="G3" s="3">
-        <v>87374</v>
+        <v>89908</v>
       </c>
       <c r="H3" s="3">
-        <v>75466</v>
+        <v>77655</v>
       </c>
     </row>
     <row r="4" spans="1:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
@@ -542,25 +542,25 @@
         <v>9</v>
       </c>
       <c r="B4" s="3">
-        <v>113048</v>
+        <v>116326</v>
       </c>
       <c r="C4" s="3">
-        <v>138452</v>
+        <v>142467</v>
       </c>
       <c r="D4" s="3">
-        <v>192385</v>
+        <v>197964</v>
       </c>
       <c r="E4" s="3">
-        <v>331617</v>
+        <v>341234</v>
       </c>
       <c r="F4" s="3">
-        <v>559044</v>
+        <v>575256</v>
       </c>
       <c r="G4" s="3">
-        <v>98189</v>
+        <v>101036</v>
       </c>
       <c r="H4" s="3">
-        <v>85123</v>
+        <v>87592</v>
       </c>
     </row>
     <row r="5" spans="1:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
@@ -568,25 +568,25 @@
         <v>10</v>
       </c>
       <c r="B5" s="3">
-        <v>159571</v>
+        <v>164199</v>
       </c>
       <c r="C5" s="3">
-        <v>228155</v>
+        <v>234771</v>
       </c>
       <c r="D5" s="3">
-        <v>267240</v>
+        <v>274990</v>
       </c>
       <c r="E5" s="3">
-        <v>447829</v>
+        <v>460816</v>
       </c>
       <c r="F5" s="3">
-        <v>666822</v>
+        <v>686160</v>
       </c>
       <c r="G5" s="3">
-        <v>139198</v>
+        <v>143235</v>
       </c>
       <c r="H5" s="3">
-        <v>121076</v>
+        <v>124587</v>
       </c>
     </row>
     <row r="6" spans="1:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
@@ -594,25 +594,25 @@
         <v>11</v>
       </c>
       <c r="B6" s="3">
-        <v>274375</v>
+        <v>282332</v>
       </c>
       <c r="C6" s="3">
-        <v>365479</v>
+        <v>376078</v>
       </c>
       <c r="D6" s="3">
-        <v>481030</v>
+        <v>494980</v>
       </c>
       <c r="E6" s="3">
-        <v>670467</v>
+        <v>689911</v>
       </c>
       <c r="F6" s="3">
-        <v>913667</v>
+        <v>940163</v>
       </c>
       <c r="G6" s="3">
-        <v>240413</v>
+        <v>247385</v>
       </c>
       <c r="H6" s="3">
-        <v>209821</v>
+        <v>215906</v>
       </c>
     </row>
     <row r="7" spans="1:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
@@ -620,25 +620,25 @@
         <v>12</v>
       </c>
       <c r="B7" s="3">
-        <v>71754</v>
+        <v>73835</v>
       </c>
       <c r="C7" s="3">
-        <v>98246</v>
+        <v>101095</v>
       </c>
       <c r="D7" s="3">
-        <v>128411</v>
+        <v>132135</v>
       </c>
       <c r="E7" s="3">
-        <v>242710</v>
+        <v>249749</v>
       </c>
       <c r="F7" s="3">
-        <v>354104</v>
+        <v>364373</v>
       </c>
       <c r="G7" s="3">
-        <v>68209</v>
+        <v>70187</v>
       </c>
       <c r="H7" s="3">
-        <v>61387</v>
+        <v>63167</v>
       </c>
     </row>
     <row r="8" spans="1:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
@@ -646,25 +646,25 @@
         <v>13</v>
       </c>
       <c r="B8" s="3">
-        <v>73100</v>
+        <v>75220</v>
       </c>
       <c r="C8" s="3">
-        <v>99217</v>
+        <v>102094</v>
       </c>
       <c r="D8" s="3">
-        <v>128371</v>
+        <v>132094</v>
       </c>
       <c r="E8" s="3">
-        <v>244709</v>
+        <v>251806</v>
       </c>
       <c r="F8" s="3">
-        <v>360677</v>
+        <v>371137</v>
       </c>
       <c r="G8" s="3">
-        <v>67883</v>
+        <v>69852</v>
       </c>
       <c r="H8" s="3">
-        <v>63358</v>
+        <v>65195</v>
       </c>
     </row>
     <row r="9" spans="1:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
@@ -672,25 +672,25 @@
         <v>14</v>
       </c>
       <c r="B9" s="3">
-        <v>83899</v>
+        <v>86332</v>
       </c>
       <c r="C9" s="3">
-        <v>112311</v>
+        <v>115568</v>
       </c>
       <c r="D9" s="3">
-        <v>148212</v>
+        <v>152510</v>
       </c>
       <c r="E9" s="3">
-        <v>283924</v>
+        <v>292158</v>
       </c>
       <c r="F9" s="3">
-        <v>416460</v>
+        <v>428537</v>
       </c>
       <c r="G9" s="3">
-        <v>79364</v>
+        <v>81666</v>
       </c>
       <c r="H9" s="3">
-        <v>74339</v>
+        <v>76495</v>
       </c>
     </row>
     <row r="10" spans="1:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
@@ -698,25 +698,25 @@
         <v>15</v>
       </c>
       <c r="B10" s="3">
-        <v>102252</v>
+        <v>105217</v>
       </c>
       <c r="C10" s="3">
-        <v>143740</v>
+        <v>147908</v>
       </c>
       <c r="D10" s="3">
-        <v>176535</v>
+        <v>181655</v>
       </c>
       <c r="E10" s="3">
-        <v>341825</v>
+        <v>351738</v>
       </c>
       <c r="F10" s="3">
-        <v>487328</v>
+        <v>501461</v>
       </c>
       <c r="G10" s="3">
-        <v>95345</v>
+        <v>98110</v>
       </c>
       <c r="H10" s="3">
-        <v>89309</v>
+        <v>91899</v>
       </c>
     </row>
     <row r="11" spans="1:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
@@ -724,25 +724,25 @@
         <v>16</v>
       </c>
       <c r="B11" s="3">
-        <v>85049</v>
+        <v>87515</v>
       </c>
       <c r="C11" s="3">
-        <v>109238</v>
+        <v>112406</v>
       </c>
       <c r="D11" s="3">
-        <v>143763</v>
+        <v>147932</v>
       </c>
       <c r="E11" s="3">
-        <v>243721</v>
+        <v>250789</v>
       </c>
       <c r="F11" s="3">
-        <v>420725</v>
+        <v>432926</v>
       </c>
       <c r="G11" s="3">
-        <v>74076</v>
+        <v>76224</v>
       </c>
       <c r="H11" s="3">
-        <v>63895</v>
+        <v>65748</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update price tables - marzo 2026
</commit_message>
<xml_diff>
--- a/cotizador.xlsx
+++ b/cotizador.xlsx
@@ -490,25 +490,25 @@
         <v>7</v>
       </c>
       <c r="B2" s="3">
-        <v>102962</v>
+        <v>105999</v>
       </c>
       <c r="C2" s="3">
-        <v>132246</v>
+        <v>136147</v>
       </c>
       <c r="D2" s="3">
-        <v>174039</v>
+        <v>179173</v>
       </c>
       <c r="E2" s="3">
-        <v>295045</v>
+        <v>303749</v>
       </c>
       <c r="F2" s="3">
-        <v>509325</v>
+        <v>524350</v>
       </c>
       <c r="G2" s="3">
-        <v>89673</v>
+        <v>92318</v>
       </c>
       <c r="H2" s="3">
-        <v>77350</v>
+        <v>79632</v>
       </c>
     </row>
     <row r="3" spans="1:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
@@ -516,25 +516,25 @@
         <v>8</v>
       </c>
       <c r="B3" s="3">
-        <v>103410</v>
+        <v>106461</v>
       </c>
       <c r="C3" s="3">
-        <v>142177</v>
+        <v>146371</v>
       </c>
       <c r="D3" s="3">
-        <v>175686</v>
+        <v>180869</v>
       </c>
       <c r="E3" s="3">
-        <v>303167</v>
+        <v>312110</v>
       </c>
       <c r="F3" s="3">
-        <v>510902</v>
+        <v>525974</v>
       </c>
       <c r="G3" s="3">
-        <v>89908</v>
+        <v>92560</v>
       </c>
       <c r="H3" s="3">
-        <v>77655</v>
+        <v>79946</v>
       </c>
     </row>
     <row r="4" spans="1:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
@@ -542,25 +542,25 @@
         <v>9</v>
       </c>
       <c r="B4" s="3">
-        <v>116326</v>
+        <v>119758</v>
       </c>
       <c r="C4" s="3">
-        <v>142467</v>
+        <v>146670</v>
       </c>
       <c r="D4" s="3">
-        <v>197964</v>
+        <v>203804</v>
       </c>
       <c r="E4" s="3">
-        <v>341234</v>
+        <v>351300</v>
       </c>
       <c r="F4" s="3">
-        <v>575256</v>
+        <v>592226</v>
       </c>
       <c r="G4" s="3">
-        <v>101036</v>
+        <v>104017</v>
       </c>
       <c r="H4" s="3">
-        <v>87592</v>
+        <v>90176</v>
       </c>
     </row>
     <row r="5" spans="1:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
@@ -568,25 +568,25 @@
         <v>10</v>
       </c>
       <c r="B5" s="3">
-        <v>164199</v>
+        <v>169043</v>
       </c>
       <c r="C5" s="3">
-        <v>234771</v>
+        <v>241697</v>
       </c>
       <c r="D5" s="3">
-        <v>274990</v>
+        <v>283102</v>
       </c>
       <c r="E5" s="3">
-        <v>460816</v>
+        <v>474410</v>
       </c>
       <c r="F5" s="3">
-        <v>686160</v>
+        <v>706402</v>
       </c>
       <c r="G5" s="3">
-        <v>143235</v>
+        <v>147460</v>
       </c>
       <c r="H5" s="3">
-        <v>124587</v>
+        <v>128262</v>
       </c>
     </row>
     <row r="6" spans="1:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
@@ -594,25 +594,25 @@
         <v>11</v>
       </c>
       <c r="B6" s="3">
-        <v>282332</v>
+        <v>290661</v>
       </c>
       <c r="C6" s="3">
-        <v>376078</v>
+        <v>387172</v>
       </c>
       <c r="D6" s="3">
-        <v>494980</v>
+        <v>509582</v>
       </c>
       <c r="E6" s="3">
-        <v>689911</v>
+        <v>710263</v>
       </c>
       <c r="F6" s="3">
-        <v>940163</v>
+        <v>967898</v>
       </c>
       <c r="G6" s="3">
-        <v>247385</v>
+        <v>254683</v>
       </c>
       <c r="H6" s="3">
-        <v>215906</v>
+        <v>222275</v>
       </c>
     </row>
     <row r="7" spans="1:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
@@ -620,25 +620,25 @@
         <v>12</v>
       </c>
       <c r="B7" s="3">
-        <v>73835</v>
+        <v>76013</v>
       </c>
       <c r="C7" s="3">
-        <v>101095</v>
+        <v>104077</v>
       </c>
       <c r="D7" s="3">
-        <v>132135</v>
+        <v>136033</v>
       </c>
       <c r="E7" s="3">
-        <v>249749</v>
+        <v>257117</v>
       </c>
       <c r="F7" s="3">
-        <v>364373</v>
+        <v>375122</v>
       </c>
       <c r="G7" s="3">
-        <v>70187</v>
+        <v>72258</v>
       </c>
       <c r="H7" s="3">
-        <v>63167</v>
+        <v>65030</v>
       </c>
     </row>
     <row r="8" spans="1:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
@@ -646,25 +646,25 @@
         <v>13</v>
       </c>
       <c r="B8" s="3">
-        <v>75220</v>
+        <v>77439</v>
       </c>
       <c r="C8" s="3">
-        <v>102094</v>
+        <v>105106</v>
       </c>
       <c r="D8" s="3">
-        <v>132094</v>
+        <v>135991</v>
       </c>
       <c r="E8" s="3">
-        <v>251806</v>
+        <v>259234</v>
       </c>
       <c r="F8" s="3">
-        <v>371137</v>
+        <v>382086</v>
       </c>
       <c r="G8" s="3">
-        <v>69852</v>
+        <v>71913</v>
       </c>
       <c r="H8" s="3">
-        <v>65195</v>
+        <v>67118</v>
       </c>
     </row>
     <row r="9" spans="1:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
@@ -672,25 +672,25 @@
         <v>14</v>
       </c>
       <c r="B9" s="3">
-        <v>86332</v>
+        <v>88879</v>
       </c>
       <c r="C9" s="3">
-        <v>115568</v>
+        <v>118977</v>
       </c>
       <c r="D9" s="3">
-        <v>152510</v>
+        <v>157009</v>
       </c>
       <c r="E9" s="3">
-        <v>292158</v>
+        <v>300777</v>
       </c>
       <c r="F9" s="3">
-        <v>428537</v>
+        <v>441179</v>
       </c>
       <c r="G9" s="3">
-        <v>81666</v>
+        <v>84075</v>
       </c>
       <c r="H9" s="3">
-        <v>76495</v>
+        <v>78752</v>
       </c>
     </row>
     <row r="10" spans="1:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
@@ -698,25 +698,25 @@
         <v>15</v>
       </c>
       <c r="B10" s="3">
-        <v>105217</v>
+        <v>108321</v>
       </c>
       <c r="C10" s="3">
-        <v>147908</v>
+        <v>152271</v>
       </c>
       <c r="D10" s="3">
-        <v>181655</v>
+        <v>187014</v>
       </c>
       <c r="E10" s="3">
-        <v>351738</v>
+        <v>362114</v>
       </c>
       <c r="F10" s="3">
-        <v>501461</v>
+        <v>516254</v>
       </c>
       <c r="G10" s="3">
-        <v>98110</v>
+        <v>101004</v>
       </c>
       <c r="H10" s="3">
-        <v>91899</v>
+        <v>94610</v>
       </c>
     </row>
     <row r="11" spans="1:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
@@ -724,25 +724,25 @@
         <v>16</v>
       </c>
       <c r="B11" s="3">
-        <v>87515</v>
+        <v>90097</v>
       </c>
       <c r="C11" s="3">
-        <v>112406</v>
+        <v>115722</v>
       </c>
       <c r="D11" s="3">
-        <v>147932</v>
+        <v>152296</v>
       </c>
       <c r="E11" s="3">
-        <v>250789</v>
+        <v>258187</v>
       </c>
       <c r="F11" s="3">
-        <v>432926</v>
+        <v>445697</v>
       </c>
       <c r="G11" s="3">
-        <v>76224</v>
+        <v>78473</v>
       </c>
       <c r="H11" s="3">
-        <v>65748</v>
+        <v>67688</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update price tables - mayo 2026
</commit_message>
<xml_diff>
--- a/cotizador.xlsx
+++ b/cotizador.xlsx
@@ -490,25 +490,25 @@
         <v>7</v>
       </c>
       <c r="B2" s="3">
-        <v>105999</v>
+        <v>109656</v>
       </c>
       <c r="C2" s="3">
-        <v>136147</v>
+        <v>140844</v>
       </c>
       <c r="D2" s="3">
-        <v>179173</v>
+        <v>185354</v>
       </c>
       <c r="E2" s="3">
-        <v>303749</v>
+        <v>314228</v>
       </c>
       <c r="F2" s="3">
-        <v>524350</v>
+        <v>542440</v>
       </c>
       <c r="G2" s="3">
-        <v>92318</v>
+        <v>95503</v>
       </c>
       <c r="H2" s="3">
-        <v>79632</v>
+        <v>82379</v>
       </c>
     </row>
     <row r="3" spans="1:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
@@ -516,25 +516,25 @@
         <v>8</v>
       </c>
       <c r="B3" s="3">
-        <v>106461</v>
+        <v>110134</v>
       </c>
       <c r="C3" s="3">
-        <v>146371</v>
+        <v>151421</v>
       </c>
       <c r="D3" s="3">
-        <v>180869</v>
+        <v>187109</v>
       </c>
       <c r="E3" s="3">
-        <v>312110</v>
+        <v>322878</v>
       </c>
       <c r="F3" s="3">
-        <v>525974</v>
+        <v>544120</v>
       </c>
       <c r="G3" s="3">
-        <v>92560</v>
+        <v>95753</v>
       </c>
       <c r="H3" s="3">
-        <v>79946</v>
+        <v>82704</v>
       </c>
     </row>
     <row r="4" spans="1:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
@@ -542,25 +542,25 @@
         <v>9</v>
       </c>
       <c r="B4" s="3">
-        <v>119758</v>
+        <v>123890</v>
       </c>
       <c r="C4" s="3">
-        <v>146670</v>
+        <v>151730</v>
       </c>
       <c r="D4" s="3">
-        <v>203804</v>
+        <v>210835</v>
       </c>
       <c r="E4" s="3">
-        <v>351300</v>
+        <v>363420</v>
       </c>
       <c r="F4" s="3">
-        <v>592226</v>
+        <v>612658</v>
       </c>
       <c r="G4" s="3">
-        <v>104017</v>
+        <v>107606</v>
       </c>
       <c r="H4" s="3">
-        <v>90176</v>
+        <v>93287</v>
       </c>
     </row>
     <row r="5" spans="1:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
@@ -568,25 +568,25 @@
         <v>10</v>
       </c>
       <c r="B5" s="3">
-        <v>169043</v>
+        <v>174875</v>
       </c>
       <c r="C5" s="3">
-        <v>241697</v>
+        <v>250036</v>
       </c>
       <c r="D5" s="3">
-        <v>283102</v>
+        <v>292869</v>
       </c>
       <c r="E5" s="3">
-        <v>474410</v>
+        <v>490777</v>
       </c>
       <c r="F5" s="3">
-        <v>706402</v>
+        <v>730773</v>
       </c>
       <c r="G5" s="3">
-        <v>147460</v>
+        <v>152547</v>
       </c>
       <c r="H5" s="3">
-        <v>128262</v>
+        <v>132687</v>
       </c>
     </row>
     <row r="6" spans="1:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
@@ -594,25 +594,25 @@
         <v>11</v>
       </c>
       <c r="B6" s="3">
-        <v>290661</v>
+        <v>300689</v>
       </c>
       <c r="C6" s="3">
-        <v>387172</v>
+        <v>400529</v>
       </c>
       <c r="D6" s="3">
-        <v>509582</v>
+        <v>527163</v>
       </c>
       <c r="E6" s="3">
-        <v>710263</v>
+        <v>734767</v>
       </c>
       <c r="F6" s="3">
-        <v>967898</v>
+        <v>1001290</v>
       </c>
       <c r="G6" s="3">
-        <v>254683</v>
+        <v>263470</v>
       </c>
       <c r="H6" s="3">
-        <v>222275</v>
+        <v>229943</v>
       </c>
     </row>
     <row r="7" spans="1:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
@@ -620,25 +620,25 @@
         <v>12</v>
       </c>
       <c r="B7" s="3">
-        <v>76013</v>
+        <v>78635</v>
       </c>
       <c r="C7" s="3">
-        <v>104077</v>
+        <v>107668</v>
       </c>
       <c r="D7" s="3">
-        <v>136033</v>
+        <v>140726</v>
       </c>
       <c r="E7" s="3">
-        <v>257117</v>
+        <v>265988</v>
       </c>
       <c r="F7" s="3">
-        <v>375122</v>
+        <v>388064</v>
       </c>
       <c r="G7" s="3">
-        <v>72258</v>
+        <v>74751</v>
       </c>
       <c r="H7" s="3">
-        <v>65030</v>
+        <v>67274</v>
       </c>
     </row>
     <row r="8" spans="1:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
@@ -646,25 +646,25 @@
         <v>13</v>
       </c>
       <c r="B8" s="3">
-        <v>77439</v>
+        <v>80111</v>
       </c>
       <c r="C8" s="3">
-        <v>105106</v>
+        <v>108732</v>
       </c>
       <c r="D8" s="3">
-        <v>135991</v>
+        <v>140683</v>
       </c>
       <c r="E8" s="3">
-        <v>259234</v>
+        <v>268178</v>
       </c>
       <c r="F8" s="3">
-        <v>382086</v>
+        <v>395268</v>
       </c>
       <c r="G8" s="3">
-        <v>71913</v>
+        <v>74394</v>
       </c>
       <c r="H8" s="3">
-        <v>67118</v>
+        <v>69434</v>
       </c>
     </row>
     <row r="9" spans="1:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
@@ -672,25 +672,25 @@
         <v>14</v>
       </c>
       <c r="B9" s="3">
-        <v>88879</v>
+        <v>91945</v>
       </c>
       <c r="C9" s="3">
-        <v>118977</v>
+        <v>123082</v>
       </c>
       <c r="D9" s="3">
-        <v>157009</v>
+        <v>162426</v>
       </c>
       <c r="E9" s="3">
-        <v>300777</v>
+        <v>311154</v>
       </c>
       <c r="F9" s="3">
-        <v>441179</v>
+        <v>456400</v>
       </c>
       <c r="G9" s="3">
-        <v>84075</v>
+        <v>86976</v>
       </c>
       <c r="H9" s="3">
-        <v>78752</v>
+        <v>81469</v>
       </c>
     </row>
     <row r="10" spans="1:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
@@ -698,25 +698,25 @@
         <v>15</v>
       </c>
       <c r="B10" s="3">
-        <v>108321</v>
+        <v>112058</v>
       </c>
       <c r="C10" s="3">
-        <v>152271</v>
+        <v>157524</v>
       </c>
       <c r="D10" s="3">
-        <v>187014</v>
+        <v>193466</v>
       </c>
       <c r="E10" s="3">
-        <v>362114</v>
+        <v>374607</v>
       </c>
       <c r="F10" s="3">
-        <v>516254</v>
+        <v>534065</v>
       </c>
       <c r="G10" s="3">
-        <v>101004</v>
+        <v>104489</v>
       </c>
       <c r="H10" s="3">
-        <v>94610</v>
+        <v>97874</v>
       </c>
     </row>
     <row r="11" spans="1:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
@@ -724,25 +724,25 @@
         <v>16</v>
       </c>
       <c r="B11" s="3">
-        <v>90097</v>
+        <v>93205</v>
       </c>
       <c r="C11" s="3">
-        <v>115722</v>
+        <v>119714</v>
       </c>
       <c r="D11" s="3">
-        <v>152296</v>
+        <v>157550</v>
       </c>
       <c r="E11" s="3">
-        <v>258187</v>
+        <v>267094</v>
       </c>
       <c r="F11" s="3">
-        <v>445697</v>
+        <v>461074</v>
       </c>
       <c r="G11" s="3">
-        <v>78473</v>
+        <v>81180</v>
       </c>
       <c r="H11" s="3">
-        <v>67688</v>
+        <v>70023</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update price tables - junio 2026
</commit_message>
<xml_diff>
--- a/cotizador.xlsx
+++ b/cotizador.xlsx
@@ -5,11 +5,11 @@
   <workbookPr defaultThemeVersion="164011"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Cecilia y Lucas\Dropbox\LUCAS PICONE OMINT\2025 OMINT OK\COTIZADOR\COTIZADOR\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://grupoomint-my.sharepoint.com/personal/lpicone_omint_com_ar/Documents/Documentos/COTIZADOR/COTIZADOR_STORE/COTIZADOR/"/>
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="20490" windowHeight="7650"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="20490" windowHeight="7500"/>
   </bookViews>
   <sheets>
     <sheet name="Hoja1" sheetId="1" r:id="rId1"/>
@@ -162,7 +162,7 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" shrinkToFit="1"/>
     </xf>
-    <xf numFmtId="164" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="164" fontId="2" fillId="0" borderId="0" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -490,25 +490,25 @@
         <v>7</v>
       </c>
       <c r="B2" s="3">
-        <v>109656</v>
+        <v>112562</v>
       </c>
       <c r="C2" s="3">
-        <v>140844</v>
+        <v>144576</v>
       </c>
       <c r="D2" s="3">
-        <v>185354</v>
+        <v>190266</v>
       </c>
       <c r="E2" s="3">
-        <v>314228</v>
+        <v>322555</v>
       </c>
       <c r="F2" s="3">
-        <v>542440</v>
+        <v>556815</v>
       </c>
       <c r="G2" s="3">
-        <v>95503</v>
+        <v>98034</v>
       </c>
       <c r="H2" s="3">
-        <v>82379</v>
+        <v>84562</v>
       </c>
     </row>
     <row r="3" spans="1:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
@@ -516,25 +516,25 @@
         <v>8</v>
       </c>
       <c r="B3" s="3">
-        <v>110134</v>
+        <v>113053</v>
       </c>
       <c r="C3" s="3">
-        <v>151421</v>
+        <v>155434</v>
       </c>
       <c r="D3" s="3">
-        <v>187109</v>
+        <v>192067</v>
       </c>
       <c r="E3" s="3">
-        <v>322878</v>
+        <v>331434</v>
       </c>
       <c r="F3" s="3">
-        <v>544120</v>
+        <v>558539</v>
       </c>
       <c r="G3" s="3">
-        <v>95753</v>
+        <v>98290</v>
       </c>
       <c r="H3" s="3">
-        <v>82704</v>
+        <v>84896</v>
       </c>
     </row>
     <row r="4" spans="1:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
@@ -542,25 +542,25 @@
         <v>9</v>
       </c>
       <c r="B4" s="3">
-        <v>123890</v>
+        <v>127173</v>
       </c>
       <c r="C4" s="3">
-        <v>151730</v>
+        <v>155751</v>
       </c>
       <c r="D4" s="3">
-        <v>210835</v>
+        <v>216422</v>
       </c>
       <c r="E4" s="3">
-        <v>363420</v>
+        <v>373051</v>
       </c>
       <c r="F4" s="3">
-        <v>612658</v>
+        <v>628893</v>
       </c>
       <c r="G4" s="3">
-        <v>107606</v>
+        <v>110458</v>
       </c>
       <c r="H4" s="3">
-        <v>93287</v>
+        <v>95759</v>
       </c>
     </row>
     <row r="5" spans="1:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
@@ -568,25 +568,25 @@
         <v>10</v>
       </c>
       <c r="B5" s="3">
-        <v>174875</v>
+        <v>179509</v>
       </c>
       <c r="C5" s="3">
-        <v>250036</v>
+        <v>256662</v>
       </c>
       <c r="D5" s="3">
-        <v>292869</v>
+        <v>300630</v>
       </c>
       <c r="E5" s="3">
-        <v>490777</v>
+        <v>503783</v>
       </c>
       <c r="F5" s="3">
-        <v>730773</v>
+        <v>750138</v>
       </c>
       <c r="G5" s="3">
-        <v>152547</v>
+        <v>156589</v>
       </c>
       <c r="H5" s="3">
-        <v>132687</v>
+        <v>136203</v>
       </c>
     </row>
     <row r="6" spans="1:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
@@ -594,25 +594,25 @@
         <v>11</v>
       </c>
       <c r="B6" s="3">
-        <v>300689</v>
+        <v>308657</v>
       </c>
       <c r="C6" s="3">
-        <v>400529</v>
+        <v>411143</v>
       </c>
       <c r="D6" s="3">
-        <v>527163</v>
+        <v>541133</v>
       </c>
       <c r="E6" s="3">
-        <v>734767</v>
+        <v>754238</v>
       </c>
       <c r="F6" s="3">
-        <v>1001290</v>
+        <v>1027824</v>
       </c>
       <c r="G6" s="3">
-        <v>263470</v>
+        <v>270452</v>
       </c>
       <c r="H6" s="3">
-        <v>229943</v>
+        <v>236036</v>
       </c>
     </row>
     <row r="7" spans="1:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
@@ -620,25 +620,25 @@
         <v>12</v>
       </c>
       <c r="B7" s="3">
-        <v>78635</v>
+        <v>80719</v>
       </c>
       <c r="C7" s="3">
-        <v>107668</v>
+        <v>110521</v>
       </c>
       <c r="D7" s="3">
-        <v>140726</v>
+        <v>144455</v>
       </c>
       <c r="E7" s="3">
-        <v>265988</v>
+        <v>273037</v>
       </c>
       <c r="F7" s="3">
-        <v>388064</v>
+        <v>398348</v>
       </c>
       <c r="G7" s="3">
-        <v>74751</v>
+        <v>76732</v>
       </c>
       <c r="H7" s="3">
-        <v>67274</v>
+        <v>69057</v>
       </c>
     </row>
     <row r="8" spans="1:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
@@ -646,25 +646,25 @@
         <v>13</v>
       </c>
       <c r="B8" s="3">
-        <v>80111</v>
+        <v>82234</v>
       </c>
       <c r="C8" s="3">
-        <v>108732</v>
+        <v>111613</v>
       </c>
       <c r="D8" s="3">
-        <v>140683</v>
+        <v>144411</v>
       </c>
       <c r="E8" s="3">
-        <v>268178</v>
+        <v>275285</v>
       </c>
       <c r="F8" s="3">
-        <v>395268</v>
+        <v>405743</v>
       </c>
       <c r="G8" s="3">
-        <v>74394</v>
+        <v>76365</v>
       </c>
       <c r="H8" s="3">
-        <v>69434</v>
+        <v>71274</v>
       </c>
     </row>
     <row r="9" spans="1:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
@@ -672,25 +672,25 @@
         <v>14</v>
       </c>
       <c r="B9" s="3">
-        <v>91945</v>
+        <v>94382</v>
       </c>
       <c r="C9" s="3">
-        <v>123082</v>
+        <v>126344</v>
       </c>
       <c r="D9" s="3">
-        <v>162426</v>
+        <v>166730</v>
       </c>
       <c r="E9" s="3">
-        <v>311154</v>
+        <v>319400</v>
       </c>
       <c r="F9" s="3">
-        <v>456400</v>
+        <v>468495</v>
       </c>
       <c r="G9" s="3">
-        <v>86976</v>
+        <v>89281</v>
       </c>
       <c r="H9" s="3">
-        <v>81469</v>
+        <v>83628</v>
       </c>
     </row>
     <row r="10" spans="1:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
@@ -698,25 +698,25 @@
         <v>15</v>
       </c>
       <c r="B10" s="3">
-        <v>112058</v>
+        <v>115028</v>
       </c>
       <c r="C10" s="3">
-        <v>157524</v>
+        <v>161698</v>
       </c>
       <c r="D10" s="3">
-        <v>193466</v>
+        <v>198593</v>
       </c>
       <c r="E10" s="3">
-        <v>374607</v>
+        <v>384534</v>
       </c>
       <c r="F10" s="3">
-        <v>534065</v>
+        <v>548218</v>
       </c>
       <c r="G10" s="3">
-        <v>104489</v>
+        <v>107258</v>
       </c>
       <c r="H10" s="3">
-        <v>97874</v>
+        <v>100468</v>
       </c>
     </row>
     <row r="11" spans="1:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
@@ -724,25 +724,25 @@
         <v>16</v>
       </c>
       <c r="B11" s="3">
-        <v>93205</v>
+        <v>95675</v>
       </c>
       <c r="C11" s="3">
-        <v>119714</v>
+        <v>122886</v>
       </c>
       <c r="D11" s="3">
-        <v>157550</v>
+        <v>161725</v>
       </c>
       <c r="E11" s="3">
-        <v>267094</v>
+        <v>274172</v>
       </c>
       <c r="F11" s="3">
-        <v>461074</v>
+        <v>473292</v>
       </c>
       <c r="G11" s="3">
-        <v>81180</v>
+        <v>83331</v>
       </c>
       <c r="H11" s="3">
-        <v>70023</v>
+        <v>71879</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update price tables - julio 2026
</commit_message>
<xml_diff>
--- a/cotizador.xlsx
+++ b/cotizador.xlsx
@@ -5,7 +5,7 @@
   <workbookPr defaultThemeVersion="164011"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://grupoomint-my.sharepoint.com/personal/lpicone_omint_com_ar/Documents/Documentos/COTIZADOR/COTIZADOR_STORE/COTIZADOR/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://grupoomint-my.sharepoint.com/personal/lpicone_omint_com_ar/Documents/COTIZADOR/COTIZADOR_STORE/COTIZADOR/"/>
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
@@ -162,7 +162,7 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" shrinkToFit="1"/>
     </xf>
-    <xf numFmtId="164" fontId="2" fillId="0" borderId="0" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -490,25 +490,25 @@
         <v>7</v>
       </c>
       <c r="B2" s="3">
-        <v>112562</v>
+        <v>115826</v>
       </c>
       <c r="C2" s="3">
-        <v>144576</v>
+        <v>148769</v>
       </c>
       <c r="D2" s="3">
-        <v>190266</v>
+        <v>195784</v>
       </c>
       <c r="E2" s="3">
-        <v>322555</v>
+        <v>331909</v>
       </c>
       <c r="F2" s="3">
-        <v>556815</v>
+        <v>572963</v>
       </c>
       <c r="G2" s="3">
-        <v>98034</v>
+        <v>100877</v>
       </c>
       <c r="H2" s="3">
-        <v>84562</v>
+        <v>87014</v>
       </c>
     </row>
     <row r="3" spans="1:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
@@ -516,25 +516,25 @@
         <v>8</v>
       </c>
       <c r="B3" s="3">
-        <v>113053</v>
+        <v>116332</v>
       </c>
       <c r="C3" s="3">
-        <v>155434</v>
+        <v>159942</v>
       </c>
       <c r="D3" s="3">
-        <v>192067</v>
+        <v>197637</v>
       </c>
       <c r="E3" s="3">
-        <v>331434</v>
+        <v>341046</v>
       </c>
       <c r="F3" s="3">
-        <v>558539</v>
+        <v>574737</v>
       </c>
       <c r="G3" s="3">
-        <v>98290</v>
+        <v>101140</v>
       </c>
       <c r="H3" s="3">
-        <v>84896</v>
+        <v>87358</v>
       </c>
     </row>
     <row r="4" spans="1:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
@@ -542,25 +542,25 @@
         <v>9</v>
       </c>
       <c r="B4" s="3">
-        <v>127173</v>
+        <v>130861</v>
       </c>
       <c r="C4" s="3">
-        <v>155751</v>
+        <v>160268</v>
       </c>
       <c r="D4" s="3">
-        <v>216422</v>
+        <v>222698</v>
       </c>
       <c r="E4" s="3">
-        <v>373051</v>
+        <v>383869</v>
       </c>
       <c r="F4" s="3">
-        <v>628893</v>
+        <v>647131</v>
       </c>
       <c r="G4" s="3">
-        <v>110458</v>
+        <v>113661</v>
       </c>
       <c r="H4" s="3">
-        <v>95759</v>
+        <v>98536</v>
       </c>
     </row>
     <row r="5" spans="1:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
@@ -568,25 +568,25 @@
         <v>10</v>
       </c>
       <c r="B5" s="3">
-        <v>179509</v>
+        <v>184715</v>
       </c>
       <c r="C5" s="3">
-        <v>256662</v>
+        <v>264105</v>
       </c>
       <c r="D5" s="3">
-        <v>300630</v>
+        <v>309348</v>
       </c>
       <c r="E5" s="3">
-        <v>503783</v>
+        <v>518393</v>
       </c>
       <c r="F5" s="3">
-        <v>750138</v>
+        <v>771892</v>
       </c>
       <c r="G5" s="3">
-        <v>156589</v>
+        <v>161130</v>
       </c>
       <c r="H5" s="3">
-        <v>136203</v>
+        <v>140153</v>
       </c>
     </row>
     <row r="6" spans="1:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
@@ -594,25 +594,25 @@
         <v>11</v>
       </c>
       <c r="B6" s="3">
-        <v>308657</v>
+        <v>317608</v>
       </c>
       <c r="C6" s="3">
-        <v>411143</v>
+        <v>423066</v>
       </c>
       <c r="D6" s="3">
-        <v>541133</v>
+        <v>556826</v>
       </c>
       <c r="E6" s="3">
-        <v>754238</v>
+        <v>776111</v>
       </c>
       <c r="F6" s="3">
-        <v>1027824</v>
+        <v>1057631</v>
       </c>
       <c r="G6" s="3">
-        <v>270452</v>
+        <v>278295</v>
       </c>
       <c r="H6" s="3">
-        <v>236036</v>
+        <v>242881</v>
       </c>
     </row>
     <row r="7" spans="1:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
@@ -620,25 +620,25 @@
         <v>12</v>
       </c>
       <c r="B7" s="3">
-        <v>80719</v>
+        <v>83060</v>
       </c>
       <c r="C7" s="3">
-        <v>110521</v>
+        <v>113726</v>
       </c>
       <c r="D7" s="3">
-        <v>144455</v>
+        <v>148644</v>
       </c>
       <c r="E7" s="3">
-        <v>273037</v>
+        <v>280955</v>
       </c>
       <c r="F7" s="3">
-        <v>398348</v>
+        <v>409900</v>
       </c>
       <c r="G7" s="3">
-        <v>76732</v>
+        <v>78957</v>
       </c>
       <c r="H7" s="3">
-        <v>69057</v>
+        <v>71060</v>
       </c>
     </row>
     <row r="8" spans="1:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
@@ -646,25 +646,25 @@
         <v>13</v>
       </c>
       <c r="B8" s="3">
-        <v>82234</v>
+        <v>84619</v>
       </c>
       <c r="C8" s="3">
-        <v>111613</v>
+        <v>114850</v>
       </c>
       <c r="D8" s="3">
-        <v>144411</v>
+        <v>148599</v>
       </c>
       <c r="E8" s="3">
-        <v>275285</v>
+        <v>283268</v>
       </c>
       <c r="F8" s="3">
-        <v>405743</v>
+        <v>417510</v>
       </c>
       <c r="G8" s="3">
-        <v>76365</v>
+        <v>78580</v>
       </c>
       <c r="H8" s="3">
-        <v>71274</v>
+        <v>73341</v>
       </c>
     </row>
     <row r="9" spans="1:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
@@ -672,25 +672,25 @@
         <v>14</v>
       </c>
       <c r="B9" s="3">
-        <v>94382</v>
+        <v>97119</v>
       </c>
       <c r="C9" s="3">
-        <v>126344</v>
+        <v>130008</v>
       </c>
       <c r="D9" s="3">
-        <v>166730</v>
+        <v>171565</v>
       </c>
       <c r="E9" s="3">
-        <v>319400</v>
+        <v>328663</v>
       </c>
       <c r="F9" s="3">
-        <v>468495</v>
+        <v>482081</v>
       </c>
       <c r="G9" s="3">
-        <v>89281</v>
+        <v>91870</v>
       </c>
       <c r="H9" s="3">
-        <v>83628</v>
+        <v>86053</v>
       </c>
     </row>
     <row r="10" spans="1:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
@@ -698,25 +698,25 @@
         <v>15</v>
       </c>
       <c r="B10" s="3">
-        <v>115028</v>
+        <v>118364</v>
       </c>
       <c r="C10" s="3">
-        <v>161698</v>
+        <v>166387</v>
       </c>
       <c r="D10" s="3">
-        <v>198593</v>
+        <v>204352</v>
       </c>
       <c r="E10" s="3">
-        <v>384534</v>
+        <v>395685</v>
       </c>
       <c r="F10" s="3">
-        <v>548218</v>
+        <v>564116</v>
       </c>
       <c r="G10" s="3">
-        <v>107258</v>
+        <v>110368</v>
       </c>
       <c r="H10" s="3">
-        <v>100468</v>
+        <v>103382</v>
       </c>
     </row>
     <row r="11" spans="1:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
@@ -724,25 +724,25 @@
         <v>16</v>
       </c>
       <c r="B11" s="3">
-        <v>95675</v>
+        <v>98450</v>
       </c>
       <c r="C11" s="3">
-        <v>122886</v>
+        <v>126450</v>
       </c>
       <c r="D11" s="3">
-        <v>161725</v>
+        <v>166415</v>
       </c>
       <c r="E11" s="3">
-        <v>274172</v>
+        <v>282123</v>
       </c>
       <c r="F11" s="3">
-        <v>473292</v>
+        <v>487017</v>
       </c>
       <c r="G11" s="3">
-        <v>83331</v>
+        <v>85748</v>
       </c>
       <c r="H11" s="3">
-        <v>71879</v>
+        <v>73963</v>
       </c>
     </row>
   </sheetData>

</xml_diff>